<commit_message>
Updated  till 22 /07 /2027
</commit_message>
<xml_diff>
--- a/OctopusSaas_26_06_2027/Test data/read.xlsx
+++ b/OctopusSaas_26_06_2027/Test data/read.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4C2F324-12B7-45F4-8566-7C1CE3AA4C28}"/>
+  <xr:revisionPtr revIDLastSave="530" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{487847B1-0404-48C1-AF40-949DD44A65EA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="673">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1435,6 +1435,637 @@
   </si>
   <si>
     <t>ballu</t>
+  </si>
+  <si>
+    <t>Website text field</t>
+  </si>
+  <si>
+    <t>Special acharcaters</t>
+  </si>
+  <si>
+    <t>furwfhi</t>
+  </si>
+  <si>
+    <t>56556</t>
+  </si>
+  <si>
+    <t>%^&amp;*</t>
+  </si>
+  <si>
+    <t>TC_49to51</t>
+  </si>
+  <si>
+    <t>Copy paste input</t>
+  </si>
+  <si>
+    <t>TC_53</t>
+  </si>
+  <si>
+    <t>Start fsical date</t>
+  </si>
+  <si>
+    <t>Business hour Text field</t>
+  </si>
+  <si>
+    <t>Start Facial date text field</t>
+  </si>
+  <si>
+    <t>TC_57to60</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>Hi</t>
+  </si>
+  <si>
+    <t>SDghh</t>
+  </si>
+  <si>
+    <t>13454</t>
+  </si>
+  <si>
+    <t>Combination</t>
+  </si>
+  <si>
+    <t>Ab12$%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doogle Review linnk
+</t>
+  </si>
+  <si>
+    <t>Special char</t>
+  </si>
+  <si>
+    <t>TC_062 to 65</t>
+  </si>
+  <si>
+    <t>DFGHJT</t>
+  </si>
+  <si>
+    <t>7895452</t>
+  </si>
+  <si>
+    <t>%^&amp;*(</t>
+  </si>
+  <si>
+    <t>Invalid input</t>
+  </si>
+  <si>
+    <t>Gh@ygy.com#</t>
+  </si>
+  <si>
+    <t>Valid Format</t>
+  </si>
+  <si>
+    <t>www.amazom.com</t>
+  </si>
+  <si>
+    <t>Satellite loaction Name</t>
+  </si>
+  <si>
+    <t>Portland41886</t>
+  </si>
+  <si>
+    <t>Satellite location Status Dropdown</t>
+  </si>
+  <si>
+    <t>TC_075</t>
+  </si>
+  <si>
+    <t>hfrbui</t>
+  </si>
+  <si>
+    <t>RegistrationNumber 1 Text field</t>
+  </si>
+  <si>
+    <t>TC_78to 80</t>
+  </si>
+  <si>
+    <t>SDFGH</t>
+  </si>
+  <si>
+    <t>34567</t>
+  </si>
+  <si>
+    <t>$^&amp;*</t>
+  </si>
+  <si>
+    <t>Tc_82 to 84</t>
+  </si>
+  <si>
+    <t>ftybu</t>
+  </si>
+  <si>
+    <t>8561</t>
+  </si>
+  <si>
+    <t>$%^*</t>
+  </si>
+  <si>
+    <t>EPA ID number text field</t>
+  </si>
+  <si>
+    <t>RTGHyhhh</t>
+  </si>
+  <si>
+    <t>852684</t>
+  </si>
+  <si>
+    <t>#$%^</t>
+  </si>
+  <si>
+    <t>TC_86to 88</t>
+  </si>
+  <si>
+    <t>Dot number field</t>
+  </si>
+  <si>
+    <t>tc_89TO91</t>
+  </si>
+  <si>
+    <t>JHGFV</t>
+  </si>
+  <si>
+    <t>865</t>
+  </si>
+  <si>
+    <t>EIN number</t>
+  </si>
+  <si>
+    <t>TC_92to94</t>
+  </si>
+  <si>
+    <t>GFhjjk</t>
+  </si>
+  <si>
+    <t>$%^&amp;*</t>
+  </si>
+  <si>
+    <t>Entity Id number</t>
+  </si>
+  <si>
+    <t>TC_095to97</t>
+  </si>
+  <si>
+    <t>Hjbj</t>
+  </si>
+  <si>
+    <t>45678</t>
+  </si>
+  <si>
+    <t>856369</t>
+  </si>
+  <si>
+    <t>SoS Numbers</t>
+  </si>
+  <si>
+    <t>TC_98to100</t>
+  </si>
+  <si>
+    <t>tfvV</t>
+  </si>
+  <si>
+    <t>3456</t>
+  </si>
+  <si>
+    <t>SIC code</t>
+  </si>
+  <si>
+    <t>TGfghj</t>
+  </si>
+  <si>
+    <t>5896</t>
+  </si>
+  <si>
+    <t>NAICS code</t>
+  </si>
+  <si>
+    <t>guib</t>
+  </si>
+  <si>
+    <t>7556</t>
+  </si>
+  <si>
+    <t>#$%^&amp;*</t>
+  </si>
+  <si>
+    <t>CAGE code</t>
+  </si>
+  <si>
+    <t>TC_101to103</t>
+  </si>
+  <si>
+    <t>TC_104to106</t>
+  </si>
+  <si>
+    <t>T107to 109</t>
+  </si>
+  <si>
+    <t>YGJ</t>
+  </si>
+  <si>
+    <t>$%^</t>
+  </si>
+  <si>
+    <t>Name text field</t>
+  </si>
+  <si>
+    <t>TC_110to112</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>84658</t>
+  </si>
+  <si>
+    <t>TC_114to116</t>
+  </si>
+  <si>
+    <t>KJN</t>
+  </si>
+  <si>
+    <t>3356</t>
+  </si>
+  <si>
+    <t>(*&amp;%^</t>
+  </si>
+  <si>
+    <t>Street text field</t>
+  </si>
+  <si>
+    <t>Valid Street Address</t>
+  </si>
+  <si>
+    <t>1237 3rd Street</t>
+  </si>
+  <si>
+    <t>Suite Text field</t>
+  </si>
+  <si>
+    <t>TC_120to122</t>
+  </si>
+  <si>
+    <t>huenf</t>
+  </si>
+  <si>
+    <t>56464</t>
+  </si>
+  <si>
+    <t>%*($%^**</t>
+  </si>
+  <si>
+    <t>City text field</t>
+  </si>
+  <si>
+    <t>Special Char</t>
+  </si>
+  <si>
+    <t>TC_124to126</t>
+  </si>
+  <si>
+    <t>lnege</t>
+  </si>
+  <si>
+    <t>987</t>
+  </si>
+  <si>
+    <t>^%$#</t>
+  </si>
+  <si>
+    <t>State Txet field</t>
+  </si>
+  <si>
+    <t>TC_129 to 131</t>
+  </si>
+  <si>
+    <t>Fcjbk</t>
+  </si>
+  <si>
+    <t>84889</t>
+  </si>
+  <si>
+    <t>Zip code text field</t>
+  </si>
+  <si>
+    <t>TC_133 to135</t>
+  </si>
+  <si>
+    <t>Iuhnjn</t>
+  </si>
+  <si>
+    <t>2616</t>
+  </si>
+  <si>
+    <t>Email Text field</t>
+  </si>
+  <si>
+    <t>TC_137to140</t>
+  </si>
+  <si>
+    <t>balli123@gmail.com</t>
+  </si>
+  <si>
+    <t>HUIhfur</t>
+  </si>
+  <si>
+    <t>43143</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid </t>
+  </si>
+  <si>
+    <t>com.@@.com</t>
+  </si>
+  <si>
+    <t>Valid mail ID</t>
+  </si>
+  <si>
+    <t>ballu123@gmail.com</t>
+  </si>
+  <si>
+    <t>Phone number Text field</t>
+  </si>
+  <si>
+    <t>TC_144 to 147</t>
+  </si>
+  <si>
+    <t>243643</t>
+  </si>
+  <si>
+    <t>hbhjbef</t>
+  </si>
+  <si>
+    <t>5646548488</t>
+  </si>
+  <si>
+    <t>$%^&amp;*(</t>
+  </si>
+  <si>
+    <t>Ext text field</t>
+  </si>
+  <si>
+    <t>Tc_149 to 152</t>
+  </si>
+  <si>
+    <t>58975</t>
+  </si>
+  <si>
+    <t>ugi</t>
+  </si>
+  <si>
+    <t>85988</t>
+  </si>
+  <si>
+    <t>&amp;^%@</t>
+  </si>
+  <si>
+    <t>More than 5 digits</t>
+  </si>
+  <si>
+    <t>134525</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Satellite Billing Information</t>
+  </si>
+  <si>
+    <t>Tc_155to 157</t>
+  </si>
+  <si>
+    <t>veggg</t>
+  </si>
+  <si>
+    <t>64864</t>
+  </si>
+  <si>
+    <t>(*^*%</t>
+  </si>
+  <si>
+    <t>Tc_159to161</t>
+  </si>
+  <si>
+    <t>urig</t>
+  </si>
+  <si>
+    <t>564894</t>
+  </si>
+  <si>
+    <t>*&amp;%#@*</t>
+  </si>
+  <si>
+    <t>TC_165 to167</t>
+  </si>
+  <si>
+    <t>bufrei</t>
+  </si>
+  <si>
+    <t>56156</t>
+  </si>
+  <si>
+    <t>%*%$%</t>
+  </si>
+  <si>
+    <t>TC169to171</t>
+  </si>
+  <si>
+    <t>cdgi</t>
+  </si>
+  <si>
+    <t>64861</t>
+  </si>
+  <si>
+    <t>%*^%^$</t>
+  </si>
+  <si>
+    <t>jhcwvdjc</t>
+  </si>
+  <si>
+    <t>684863</t>
+  </si>
+  <si>
+    <t>(&amp;(*&amp;^%</t>
+  </si>
+  <si>
+    <t>Tc_173 to 175</t>
+  </si>
+  <si>
+    <t>TC_177 to 179</t>
+  </si>
+  <si>
+    <t>kjhrwiug</t>
+  </si>
+  <si>
+    <t>86969</t>
+  </si>
+  <si>
+    <t>#$%^*(</t>
+  </si>
+  <si>
+    <t>Valid Input</t>
+  </si>
+  <si>
+    <t>TC_181 to 184</t>
+  </si>
+  <si>
+    <t>charlie123@gmail.com</t>
+  </si>
+  <si>
+    <t>GYJgj</t>
+  </si>
+  <si>
+    <t>547831</t>
+  </si>
+  <si>
+    <t>&amp;*%8758</t>
+  </si>
+  <si>
+    <t>TC_188 to 191</t>
+  </si>
+  <si>
+    <t>5897458962</t>
+  </si>
+  <si>
+    <t>jjkwbv</t>
+  </si>
+  <si>
+    <t>1234568759</t>
+  </si>
+  <si>
+    <t>*%8758</t>
+  </si>
+  <si>
+    <t>invalid format</t>
+  </si>
+  <si>
+    <t>Tc_194 to 199</t>
+  </si>
+  <si>
+    <t>58945</t>
+  </si>
+  <si>
+    <t>fedsvs</t>
+  </si>
+  <si>
+    <t>68454</t>
+  </si>
+  <si>
+    <t>^$&amp;*&amp;</t>
+  </si>
+  <si>
+    <t>589745</t>
+  </si>
+  <si>
+    <t>Valid name</t>
+  </si>
+  <si>
+    <t>Naren</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>90210</t>
+  </si>
+  <si>
+    <t>Exact Phone Number</t>
+  </si>
+  <si>
+    <t>8596478598</t>
+  </si>
+  <si>
+    <t>Dispatch Department</t>
+  </si>
+  <si>
+    <t>invalid input</t>
+  </si>
+  <si>
+    <t>TC_211 to215</t>
+  </si>
+  <si>
+    <t>jcwdc</t>
+  </si>
+  <si>
+    <t>657897</t>
+  </si>
+  <si>
+    <t>&amp;%&amp;$%#</t>
+  </si>
+  <si>
+    <t>.com@.com</t>
+  </si>
+  <si>
+    <t>TC_217to220</t>
+  </si>
+  <si>
+    <t>9305948592</t>
+  </si>
+  <si>
+    <t>wufifrwf</t>
+  </si>
+  <si>
+    <t>23434242433</t>
+  </si>
+  <si>
+    <t>*(&amp;(^*&amp;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special char </t>
+  </si>
+  <si>
+    <t>jhqvfew</t>
+  </si>
+  <si>
+    <t>58963</t>
+  </si>
+  <si>
+    <t>%&amp;**%$</t>
+  </si>
+  <si>
+    <t>589632</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>TC_222to228</t>
+  </si>
+  <si>
+    <t>Comapany Display Name</t>
+  </si>
+  <si>
+    <t>Registration number 1</t>
+  </si>
+  <si>
+    <t>General information fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portland </t>
+  </si>
+  <si>
+    <t>5897412563</t>
+  </si>
+  <si>
+    <t>698742</t>
+  </si>
+  <si>
+    <t>Tc_228</t>
+  </si>
+  <si>
+    <t>Dispatch email</t>
+  </si>
+  <si>
+    <t>Dispatch phone</t>
+  </si>
+  <si>
+    <t>naren</t>
+  </si>
+  <si>
+    <t>5896321475</t>
   </si>
 </sst>
 </file>
@@ -1458,7 +2089,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1468,6 +2099,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1485,7 +2122,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -1504,6 +2141,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3922,15 +4562,18 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
     <col min="2" max="2" width="25" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="6"/>
-    <col min="4" max="4" width="15.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="18.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
@@ -4082,7 +4725,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>445</v>
       </c>
@@ -4116,7 +4759,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="4" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" s="4" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>450</v>
       </c>
@@ -4173,6 +4816,1238 @@
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B25" s="6" t="s">
         <v>462</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>478</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="4" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>485</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>503</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>507</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>513</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>529</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>543</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A62" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>546</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>554</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>569</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A72" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A73" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>572</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A74" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A75" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>583</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="F75" s="8" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>590</v>
+      </c>
+      <c r="F77" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" s="10" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>597</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>601</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>612</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A91" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="B92" s="9" t="s">
+        <v>621</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="G92" s="9" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A93" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>626</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>628</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A95" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>632</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="D96" s="8" t="s">
+        <v>634</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>636</v>
+      </c>
+      <c r="G96" s="8" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" s="10" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A98" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>644</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>621</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>647</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>649</v>
+      </c>
+      <c r="G99" s="9" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>651</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>655</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="D103" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>659</v>
+      </c>
+      <c r="G103" s="8" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A105" s="4" t="s">
+        <v>664</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>666</v>
+      </c>
+      <c r="D106" s="8" t="s">
+        <v>667</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>672</v>
       </c>
     </row>
   </sheetData>
@@ -4181,6 +6056,19 @@
     <hyperlink ref="B6" r:id="rId2" xr:uid="{284322BF-D005-4BF8-9C8A-1D78ADDFD986}"/>
     <hyperlink ref="E6" r:id="rId3" xr:uid="{77471F4F-AA24-4166-BB1C-7C0B003FB5F7}"/>
     <hyperlink ref="B10" r:id="rId4" xr:uid="{A5A7610F-A733-45B6-90BA-72F05DA28534}"/>
+    <hyperlink ref="E28" r:id="rId5" xr:uid="{1269199C-B882-4CF4-8FE7-B5632B815114}"/>
+    <hyperlink ref="B36" r:id="rId6" xr:uid="{F80053D1-6192-46D4-8135-3162E9DCDBFF}"/>
+    <hyperlink ref="F36" r:id="rId7" xr:uid="{A2E87AD7-519E-4D64-A8B0-804F45B567E3}"/>
+    <hyperlink ref="G36" r:id="rId8" xr:uid="{001C606C-950A-42AD-84B8-A6A9B9513EE9}"/>
+    <hyperlink ref="B73" r:id="rId9" xr:uid="{24CFF544-36E4-4F50-A277-C01ABB4FEEC2}"/>
+    <hyperlink ref="F73" r:id="rId10" display="com@" xr:uid="{C8CFEF57-B152-49C3-AFFA-70B8D30BAEEE}"/>
+    <hyperlink ref="G73" r:id="rId11" xr:uid="{ACEECA67-88F7-427D-BFAF-783DE7661C96}"/>
+    <hyperlink ref="E77" r:id="rId12" xr:uid="{4E986B8C-EDF0-45DA-B387-2BAFD2E8026F}"/>
+    <hyperlink ref="D82" r:id="rId13" xr:uid="{CDD6978D-1DF9-47A7-99E0-AA10BDC906A5}"/>
+    <hyperlink ref="B92" r:id="rId14" xr:uid="{15FDAB5F-0AF4-4F79-8B5D-CA436D3B9DC1}"/>
+    <hyperlink ref="G92" r:id="rId15" xr:uid="{224A48AA-0076-41B6-B0C3-F943D56C406C}"/>
+    <hyperlink ref="F99" r:id="rId16" xr:uid="{10706437-A8D3-431D-AB38-0D11EC24B8B2}"/>
+    <hyperlink ref="G99" r:id="rId17" display="charlie123@gmail.com" xr:uid="{BE1272E6-3091-460B-92B3-2F7568D11C99}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>